<commit_message>
teste de dunn e correções
</commit_message>
<xml_diff>
--- a/databases/mann_kendall_taxa_por_1000_mulheres.xlsx
+++ b/databases/mann_kendall_taxa_por_1000_mulheres.xlsx
@@ -414,12 +414,10 @@
         <v>6.4</v>
       </c>
       <c r="D2">
-        <v>-3.34</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>8e-04</t>
-        </is>
+        <v>-3.3404</v>
+      </c>
+      <c r="E2">
+        <v>0.0008</v>
       </c>
       <c r="F2">
         <v>7.1</v>
@@ -428,12 +426,10 @@
         <v>5.1</v>
       </c>
       <c r="H2">
-        <v>-2.351</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.0187</t>
-        </is>
+        <v>-2.3506</v>
+      </c>
+      <c r="I2">
+        <v>0.0187</v>
       </c>
     </row>
     <row r="3">
@@ -449,12 +445,10 @@
         <v>14</v>
       </c>
       <c r="D3">
-        <v>-0.619</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0.5362</t>
-        </is>
+        <v>-0.6186</v>
+      </c>
+      <c r="E3">
+        <v>0.5362</v>
       </c>
       <c r="F3">
         <v>1.9</v>
@@ -463,12 +457,10 @@
         <v>1.4</v>
       </c>
       <c r="H3">
-        <v>-1.634</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.1024</t>
-        </is>
+        <v>-1.6335</v>
+      </c>
+      <c r="I3">
+        <v>0.1024</v>
       </c>
     </row>
     <row r="4">
@@ -484,12 +476,10 @@
         <v>7</v>
       </c>
       <c r="D4">
-        <v>-3.093</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
+        <v>-3.0929</v>
+      </c>
+      <c r="E4">
+        <v>0.002</v>
       </c>
       <c r="F4">
         <v>6.2</v>
@@ -498,12 +488,10 @@
         <v>4</v>
       </c>
       <c r="H4">
-        <v>-0.499</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.618</t>
-        </is>
+        <v>-0.4987</v>
+      </c>
+      <c r="I4">
+        <v>0.618</v>
       </c>
     </row>
     <row r="5">
@@ -519,12 +507,10 @@
         <v>13.1</v>
       </c>
       <c r="D5">
-        <v>-2.846</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
+        <v>-2.8455</v>
+      </c>
+      <c r="E5">
+        <v>0.0044</v>
       </c>
       <c r="F5">
         <v>4.9</v>
@@ -533,12 +519,10 @@
         <v>1.6</v>
       </c>
       <c r="H5">
-        <v>-2.598</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.0094</t>
-        </is>
+        <v>-2.5981</v>
+      </c>
+      <c r="I5">
+        <v>0.0094</v>
       </c>
     </row>
     <row r="6">
@@ -554,12 +538,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="D6">
-        <v>-2.846</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
+        <v>-2.8455</v>
+      </c>
+      <c r="E6">
+        <v>0.0044</v>
       </c>
       <c r="F6">
         <v>1.8</v>
@@ -568,12 +550,10 @@
         <v>1.4</v>
       </c>
       <c r="H6">
-        <v>-0.748</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.4544</t>
-        </is>
+        <v>-0.7481</v>
+      </c>
+      <c r="I6">
+        <v>0.4544</v>
       </c>
     </row>
     <row r="7">
@@ -589,12 +569,10 @@
         <v>8.300000000000001</v>
       </c>
       <c r="D7">
-        <v>-3.34</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>8e-04</t>
-        </is>
+        <v>-3.3404</v>
+      </c>
+      <c r="E7">
+        <v>0.0008</v>
       </c>
       <c r="F7">
         <v>5.8</v>
@@ -603,12 +581,10 @@
         <v>2.5</v>
       </c>
       <c r="H7">
-        <v>-1.885</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.0595</t>
-        </is>
+        <v>-1.8848</v>
+      </c>
+      <c r="I7">
+        <v>0.0595</v>
       </c>
     </row>
     <row r="8">
@@ -624,12 +600,10 @@
         <v>7.9</v>
       </c>
       <c r="D8">
-        <v>-3.093</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
+        <v>-3.0929</v>
+      </c>
+      <c r="E8">
+        <v>0.002</v>
       </c>
       <c r="F8">
         <v>6.4</v>
@@ -638,12 +612,10 @@
         <v>3.8</v>
       </c>
       <c r="H8">
-        <v>-0.499</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.618</t>
-        </is>
+        <v>-0.4987</v>
+      </c>
+      <c r="I8">
+        <v>0.618</v>
       </c>
     </row>
     <row r="9">
@@ -659,12 +631,10 @@
         <v>5.5</v>
       </c>
       <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>-0</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
       </c>
       <c r="F9">
         <v>6.2</v>
@@ -673,12 +643,10 @@
         <v>5.6</v>
       </c>
       <c r="H9">
-        <v>0.371</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.7105</t>
-        </is>
+        <v>0.3712</v>
+      </c>
+      <c r="I9">
+        <v>0.7105</v>
       </c>
     </row>
     <row r="10">
@@ -694,12 +662,10 @@
         <v>6.4</v>
       </c>
       <c r="D10">
-        <v>-3.141</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0.0017</t>
-        </is>
+        <v>-3.1414</v>
+      </c>
+      <c r="E10">
+        <v>0.0017</v>
       </c>
       <c r="F10">
         <v>11.2</v>
@@ -708,12 +674,10 @@
         <v>5.3</v>
       </c>
       <c r="H10">
-        <v>-3.242</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.0012</t>
-        </is>
+        <v>-3.2416</v>
+      </c>
+      <c r="I10">
+        <v>0.0012</v>
       </c>
     </row>
     <row r="11">
@@ -729,12 +693,10 @@
         <v>4.8</v>
       </c>
       <c r="D11">
-        <v>-2.387</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>0.017</t>
-        </is>
+        <v>-2.3875</v>
+      </c>
+      <c r="E11">
+        <v>0.017</v>
       </c>
       <c r="F11">
         <v>6.7</v>
@@ -743,12 +705,10 @@
         <v>5.4</v>
       </c>
       <c r="H11">
-        <v>0.126</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
+        <v>0.1257</v>
+      </c>
+      <c r="I11">
+        <v>0.9</v>
       </c>
     </row>
     <row r="12">
@@ -764,12 +724,10 @@
         <v>10.2</v>
       </c>
       <c r="D12">
-        <v>-1.608</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0.1078</t>
-        </is>
+        <v>-1.6083</v>
+      </c>
+      <c r="E12">
+        <v>0.1078</v>
       </c>
       <c r="F12">
         <v>2.8</v>
@@ -778,12 +736,10 @@
         <v>3</v>
       </c>
       <c r="H12">
-        <v>1.361</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.1736</t>
-        </is>
+        <v>1.3609</v>
+      </c>
+      <c r="I12">
+        <v>0.1735</v>
       </c>
     </row>
     <row r="13">
@@ -799,12 +755,10 @@
         <v>6.1</v>
       </c>
       <c r="D13">
-        <v>0.509</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>0.6105</t>
-        </is>
+        <v>0.5094</v>
+      </c>
+      <c r="E13">
+        <v>0.6105</v>
       </c>
       <c r="F13">
         <v>6.2</v>
@@ -813,12 +767,10 @@
         <v>6.8</v>
       </c>
       <c r="H13">
-        <v>1.745</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.0809</t>
-        </is>
+        <v>1.7455</v>
+      </c>
+      <c r="I13">
+        <v>0.0809</v>
       </c>
     </row>
     <row r="14">
@@ -834,12 +786,10 @@
         <v>5.3</v>
       </c>
       <c r="D14">
-        <v>-2.846</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
+        <v>-2.8455</v>
+      </c>
+      <c r="E14">
+        <v>0.0044</v>
       </c>
       <c r="F14">
         <v>6.7</v>
@@ -848,12 +798,10 @@
         <v>7.1</v>
       </c>
       <c r="H14">
-        <v>0.619</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>0.5362</t>
-        </is>
+        <v>0.6186</v>
+      </c>
+      <c r="I14">
+        <v>0.5362</v>
       </c>
     </row>
     <row r="15">
@@ -869,12 +817,10 @@
         <v>5.4</v>
       </c>
       <c r="D15">
-        <v>-3.34</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>8e-04</t>
-        </is>
+        <v>-3.3404</v>
+      </c>
+      <c r="E15">
+        <v>0.0008</v>
       </c>
       <c r="F15">
         <v>8.1</v>
@@ -883,12 +829,10 @@
         <v>6.2</v>
       </c>
       <c r="H15">
-        <v>-2.696</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>0.007</t>
-        </is>
+        <v>-2.6962</v>
+      </c>
+      <c r="I15">
+        <v>0.007</v>
       </c>
     </row>
     <row r="16">
@@ -904,12 +848,10 @@
         <v>3.9</v>
       </c>
       <c r="D16">
-        <v>-2.89</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>0.0039</t>
-        </is>
+        <v>-2.8901</v>
+      </c>
+      <c r="E16">
+        <v>0.0039</v>
       </c>
       <c r="F16">
         <v>7.1</v>
@@ -918,12 +860,10 @@
         <v>5.8</v>
       </c>
       <c r="H16">
-        <v>-0.88</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0.3791</t>
-        </is>
+        <v>-0.8796</v>
+      </c>
+      <c r="I16">
+        <v>0.3791</v>
       </c>
     </row>
     <row r="17">
@@ -939,12 +879,10 @@
         <v>7.7</v>
       </c>
       <c r="D17">
-        <v>-2.846</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
+        <v>-2.8455</v>
+      </c>
+      <c r="E17">
+        <v>0.0044</v>
       </c>
       <c r="F17">
         <v>6.3</v>
@@ -953,12 +891,10 @@
         <v>5</v>
       </c>
       <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>-0</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -974,12 +910,10 @@
         <v>8.1</v>
       </c>
       <c r="D18">
-        <v>-3.093</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
+        <v>-3.0929</v>
+      </c>
+      <c r="E18">
+        <v>0.002</v>
       </c>
       <c r="F18">
         <v>2.5</v>
@@ -988,12 +922,10 @@
         <v>2</v>
       </c>
       <c r="H18">
-        <v>-0.507</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0.6124</t>
-        </is>
+        <v>-0.5066000000000001</v>
+      </c>
+      <c r="I18">
+        <v>0.6124000000000001</v>
       </c>
     </row>
     <row r="19">
@@ -1009,12 +941,10 @@
         <v>8.300000000000001</v>
       </c>
       <c r="D19">
-        <v>-3.093</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
+        <v>-3.0929</v>
+      </c>
+      <c r="E19">
+        <v>0.002</v>
       </c>
       <c r="F19">
         <v>4.9</v>
@@ -1023,12 +953,10 @@
         <v>2.4</v>
       </c>
       <c r="H19">
-        <v>-1.885</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0.0595</t>
-        </is>
+        <v>-1.8848</v>
+      </c>
+      <c r="I19">
+        <v>0.0595</v>
       </c>
     </row>
     <row r="20">
@@ -1044,12 +972,10 @@
         <v>7.8</v>
       </c>
       <c r="D20">
-        <v>-2.846</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
+        <v>-2.8455</v>
+      </c>
+      <c r="E20">
+        <v>0.0044</v>
       </c>
       <c r="F20">
         <v>6.1</v>
@@ -1058,12 +984,10 @@
         <v>3.3</v>
       </c>
       <c r="H20">
-        <v>-1.247</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>0.2125</t>
-        </is>
+        <v>-1.2468</v>
+      </c>
+      <c r="I20">
+        <v>0.2125</v>
       </c>
     </row>
     <row r="21">
@@ -1079,12 +1003,10 @@
         <v>6.5</v>
       </c>
       <c r="D21">
-        <v>-2.992</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>0.0028</t>
-        </is>
+        <v>-2.9922</v>
+      </c>
+      <c r="E21">
+        <v>0.0028</v>
       </c>
       <c r="F21">
         <v>6.3</v>
@@ -1093,12 +1015,10 @@
         <v>4.9</v>
       </c>
       <c r="H21">
-        <v>-0.249</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>0.8031</t>
-        </is>
+        <v>-0.2494</v>
+      </c>
+      <c r="I21">
+        <v>0.8031</v>
       </c>
     </row>
     <row r="22">
@@ -1114,12 +1034,10 @@
         <v>4.7</v>
       </c>
       <c r="D22">
-        <v>-2.598</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>0.0094</t>
-        </is>
+        <v>-2.5981</v>
+      </c>
+      <c r="E22">
+        <v>0.0094</v>
       </c>
       <c r="F22">
         <v>2.7</v>
@@ -1128,12 +1046,10 @@
         <v>3.1</v>
       </c>
       <c r="H22">
-        <v>2.244</v>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>0.0248</t>
-        </is>
+        <v>2.2442</v>
+      </c>
+      <c r="I22">
+        <v>0.0248</v>
       </c>
     </row>
     <row r="23">
@@ -1149,12 +1065,10 @@
         <v>6.5</v>
       </c>
       <c r="D23">
-        <v>-2.992</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0.0028</t>
-        </is>
+        <v>-2.9922</v>
+      </c>
+      <c r="E23">
+        <v>0.0028</v>
       </c>
       <c r="F23">
         <v>8.199999999999999</v>
@@ -1163,12 +1077,10 @@
         <v>5.7</v>
       </c>
       <c r="H23">
-        <v>-2.244</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>0.0248</t>
-        </is>
+        <v>-2.2442</v>
+      </c>
+      <c r="I23">
+        <v>0.0248</v>
       </c>
     </row>
     <row r="24">
@@ -1184,12 +1096,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="D24">
-        <v>-2.387</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0.017</t>
-        </is>
+        <v>-2.3875</v>
+      </c>
+      <c r="E24">
+        <v>0.017</v>
       </c>
       <c r="F24">
         <v>6.7</v>
@@ -1198,12 +1108,10 @@
         <v>3.7</v>
       </c>
       <c r="H24">
-        <v>-1.856</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>0.0635</t>
-        </is>
+        <v>-1.8558</v>
+      </c>
+      <c r="I24">
+        <v>0.0635</v>
       </c>
     </row>
     <row r="25">
@@ -1219,12 +1127,10 @@
         <v>6.3</v>
       </c>
       <c r="D25">
-        <v>-3.093</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
+        <v>-3.0929</v>
+      </c>
+      <c r="E25">
+        <v>0.002</v>
       </c>
       <c r="F25">
         <v>2.1</v>
@@ -1233,12 +1139,10 @@
         <v>1.4</v>
       </c>
       <c r="H25">
-        <v>-0.371</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>0.7105</t>
-        </is>
+        <v>-0.3712</v>
+      </c>
+      <c r="I25">
+        <v>0.7105</v>
       </c>
     </row>
     <row r="26">
@@ -1254,12 +1158,10 @@
         <v>5.5</v>
       </c>
       <c r="D26">
-        <v>-2.387</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>0.017</t>
-        </is>
+        <v>-2.3875</v>
+      </c>
+      <c r="E26">
+        <v>0.017</v>
       </c>
       <c r="F26">
         <v>5.9</v>
@@ -1268,12 +1170,10 @@
         <v>6.6</v>
       </c>
       <c r="H26">
-        <v>1.528</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>0.1265</t>
-        </is>
+        <v>1.5281</v>
+      </c>
+      <c r="I26">
+        <v>0.1265</v>
       </c>
     </row>
     <row r="27">
@@ -1289,12 +1189,10 @@
         <v>8</v>
       </c>
       <c r="D27">
-        <v>-3.242</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>0.0012</t>
-        </is>
+        <v>-3.2416</v>
+      </c>
+      <c r="E27">
+        <v>0.0012</v>
       </c>
       <c r="F27">
         <v>5.9</v>
@@ -1305,10 +1203,8 @@
       <c r="H27">
         <v>-0.866</v>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>0.3865</t>
-        </is>
+      <c r="I27">
+        <v>0.3865</v>
       </c>
     </row>
     <row r="28">
@@ -1324,12 +1220,10 @@
         <v>5.2</v>
       </c>
       <c r="D28">
-        <v>-3.34</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>8e-04</t>
-        </is>
+        <v>-3.3404</v>
+      </c>
+      <c r="E28">
+        <v>0.0008</v>
       </c>
       <c r="F28">
         <v>11</v>
@@ -1338,12 +1232,10 @@
         <v>7.7</v>
       </c>
       <c r="H28">
-        <v>-3.242</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>0.0012</t>
-        </is>
+        <v>-3.2416</v>
+      </c>
+      <c r="I28">
+        <v>0.0012</v>
       </c>
     </row>
     <row r="29">
@@ -1359,12 +1251,10 @@
         <v>7.2</v>
       </c>
       <c r="D29">
-        <v>-2.846</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>0.0044</t>
-        </is>
+        <v>-2.8455</v>
+      </c>
+      <c r="E29">
+        <v>0.0044</v>
       </c>
       <c r="F29">
         <v>2.6</v>
@@ -1373,12 +1263,10 @@
         <v>4.1</v>
       </c>
       <c r="H29">
-        <v>0.628</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>0.5298</t>
-        </is>
+        <v>0.6283</v>
+      </c>
+      <c r="I29">
+        <v>0.5298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correção dos dados tabnet
</commit_message>
<xml_diff>
--- a/databases/mann_kendall_taxa_por_1000_mulheres.xlsx
+++ b/databases/mann_kendall_taxa_por_1000_mulheres.xlsx
@@ -411,7 +411,7 @@
         <v>9.6</v>
       </c>
       <c r="C2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="D2">
         <v>-3.3404</v>
@@ -445,10 +445,10 @@
         <v>14</v>
       </c>
       <c r="D3">
-        <v>-0.6186</v>
+        <v>-0.866</v>
       </c>
       <c r="E3">
-        <v>0.5362</v>
+        <v>0.3865</v>
       </c>
       <c r="F3">
         <v>1.9</v>
@@ -631,10 +631,10 @@
         <v>5.5</v>
       </c>
       <c r="D9">
-        <v>-0</v>
+        <v>-0.4987</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0.618</v>
       </c>
       <c r="F9">
         <v>6.2</v>
@@ -643,10 +643,10 @@
         <v>5.6</v>
       </c>
       <c r="H9">
-        <v>0.3712</v>
+        <v>0.1237</v>
       </c>
       <c r="I9">
-        <v>0.7105</v>
+        <v>0.9015</v>
       </c>
     </row>
     <row r="10">
@@ -662,10 +662,10 @@
         <v>6.4</v>
       </c>
       <c r="D10">
-        <v>-3.1414</v>
+        <v>-2.9922</v>
       </c>
       <c r="E10">
-        <v>0.0017</v>
+        <v>0.0028</v>
       </c>
       <c r="F10">
         <v>11.2</v>
@@ -705,10 +705,10 @@
         <v>5.4</v>
       </c>
       <c r="H11">
-        <v>0.1257</v>
+        <v>-0</v>
       </c>
       <c r="I11">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -755,10 +755,10 @@
         <v>6.1</v>
       </c>
       <c r="D13">
-        <v>0.5094</v>
+        <v>0.2494</v>
       </c>
       <c r="E13">
-        <v>0.6105</v>
+        <v>0.8031</v>
       </c>
       <c r="F13">
         <v>6.2</v>
@@ -786,10 +786,10 @@
         <v>5.3</v>
       </c>
       <c r="D14">
-        <v>-2.8455</v>
+        <v>-2.9922</v>
       </c>
       <c r="E14">
-        <v>0.0044</v>
+        <v>0.0028</v>
       </c>
       <c r="F14">
         <v>6.7</v>
@@ -814,7 +814,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="C15">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="D15">
         <v>-3.3404</v>
@@ -860,10 +860,10 @@
         <v>5.8</v>
       </c>
       <c r="H16">
-        <v>-0.8796</v>
+        <v>-0.9974</v>
       </c>
       <c r="I16">
-        <v>0.3791</v>
+        <v>0.3186</v>
       </c>
     </row>
     <row r="17">
@@ -1015,10 +1015,10 @@
         <v>4.9</v>
       </c>
       <c r="H21">
-        <v>-0.2494</v>
+        <v>-0.3712</v>
       </c>
       <c r="I21">
-        <v>0.8031</v>
+        <v>0.7105</v>
       </c>
     </row>
     <row r="22">
@@ -1046,10 +1046,10 @@
         <v>3.1</v>
       </c>
       <c r="H22">
-        <v>2.2442</v>
+        <v>2.1362</v>
       </c>
       <c r="I22">
-        <v>0.0248</v>
+        <v>0.0327</v>
       </c>
     </row>
     <row r="23">
@@ -1065,10 +1065,10 @@
         <v>6.5</v>
       </c>
       <c r="D23">
-        <v>-2.9922</v>
+        <v>-2.7429</v>
       </c>
       <c r="E23">
-        <v>0.0028</v>
+        <v>0.0061</v>
       </c>
       <c r="F23">
         <v>8.199999999999999</v>
@@ -1096,10 +1096,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="D24">
-        <v>-2.3875</v>
+        <v>-2.6388</v>
       </c>
       <c r="E24">
-        <v>0.017</v>
+        <v>0.0083</v>
       </c>
       <c r="F24">
         <v>6.7</v>
@@ -1158,10 +1158,10 @@
         <v>5.5</v>
       </c>
       <c r="D26">
-        <v>-2.3875</v>
+        <v>-2.8901</v>
       </c>
       <c r="E26">
-        <v>0.017</v>
+        <v>0.0039</v>
       </c>
       <c r="F26">
         <v>5.9</v>
@@ -1170,10 +1170,10 @@
         <v>6.6</v>
       </c>
       <c r="H26">
-        <v>1.5281</v>
+        <v>1.4961</v>
       </c>
       <c r="I26">
-        <v>0.1265</v>
+        <v>0.1346</v>
       </c>
     </row>
     <row r="27">
@@ -1263,10 +1263,10 @@
         <v>4.1</v>
       </c>
       <c r="H29">
-        <v>0.6283</v>
+        <v>0.76</v>
       </c>
       <c r="I29">
-        <v>0.5298</v>
+        <v>0.4473</v>
       </c>
     </row>
   </sheetData>

</xml_diff>